<commit_message>
excel okuma ve yazma methodu eklendi.
excel okuma ve yazma methodu eklendi.
</commit_message>
<xml_diff>
--- a/EKYNOX_HOSPITAL_EXCEL_IMPORTER/EKYNOX_HEI.DAPP/Files/Extension/Temp.xlsx
+++ b/EKYNOX_HOSPITAL_EXCEL_IMPORTER/EKYNOX_HEI.DAPP/Files/Extension/Temp.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\muhar\OneDrive\Masaüstü\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\EKYNOX\EKYNOX_HOSPITAL_EXCEL_IMPORTER\EKYNOX_HOSPITAL_EXCEL_IMPORTER\EKYNOX_HEI.DAPP\Files\Extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE39E6AE-7ECE-4E02-83BF-097220DDD78F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03218337-1090-48D0-B3E9-F2DEE5F1C366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="175">
   <si>
     <t>Ad</t>
   </si>
@@ -82,9 +82,6 @@
     <t>5.Eğitim Tarihi</t>
   </si>
   <si>
-    <t>6.Eğitim</t>
-  </si>
-  <si>
     <t>7.Eğitim</t>
   </si>
   <si>
@@ -584,153 +581,6 @@
   </si>
   <si>
     <t>Kılıç</t>
-  </si>
-  <si>
-    <t>ŞAFAK</t>
-  </si>
-  <si>
-    <t>KEBABÇI</t>
-  </si>
-  <si>
-    <t>FİLİZ</t>
-  </si>
-  <si>
-    <t>YEŞİLDİŞ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DAMLA </t>
-  </si>
-  <si>
-    <t>BÜYÜKKARA</t>
-  </si>
-  <si>
-    <t>ŞİFANUR</t>
-  </si>
-  <si>
-    <t>SAYRAN</t>
-  </si>
-  <si>
-    <t>DİLEK</t>
-  </si>
-  <si>
-    <t>İPLİ</t>
-  </si>
-  <si>
-    <t>ELİF</t>
-  </si>
-  <si>
-    <t>ARICAN</t>
-  </si>
-  <si>
-    <t>NİHAL</t>
-  </si>
-  <si>
-    <t>YAZICI</t>
-  </si>
-  <si>
-    <t>ELİFNUR</t>
-  </si>
-  <si>
-    <t>DEMİRTAŞ</t>
-  </si>
-  <si>
-    <t>GİZEM</t>
-  </si>
-  <si>
-    <t>ŞEKERCİ</t>
-  </si>
-  <si>
-    <t>CEMİLE</t>
-  </si>
-  <si>
-    <t>EDA</t>
-  </si>
-  <si>
-    <t>ŞENTÜRK</t>
-  </si>
-  <si>
-    <t>İLAYDA</t>
-  </si>
-  <si>
-    <t>YALÇINKAYA</t>
-  </si>
-  <si>
-    <t>BİRSEN</t>
-  </si>
-  <si>
-    <t>US</t>
-  </si>
-  <si>
-    <t>MERYEM</t>
-  </si>
-  <si>
-    <t>YÜKSEL DİLARA</t>
-  </si>
-  <si>
-    <t>TEMEL</t>
-  </si>
-  <si>
-    <t>ALEYNA BUSE</t>
-  </si>
-  <si>
-    <t>BULUT</t>
-  </si>
-  <si>
-    <t>İREM</t>
-  </si>
-  <si>
-    <t>APALAK</t>
-  </si>
-  <si>
-    <t>MELİKE</t>
-  </si>
-  <si>
-    <t>GÜLSOY</t>
-  </si>
-  <si>
-    <t>HASİBE</t>
-  </si>
-  <si>
-    <t>BÜŞRA</t>
-  </si>
-  <si>
-    <t>YAKAR</t>
-  </si>
-  <si>
-    <t>KISMET</t>
-  </si>
-  <si>
-    <t>YILDIRIM</t>
-  </si>
-  <si>
-    <t>KAPLAN</t>
-  </si>
-  <si>
-    <t>İKRA</t>
-  </si>
-  <si>
-    <t>TUNÇ</t>
-  </si>
-  <si>
-    <t>ECEM</t>
-  </si>
-  <si>
-    <t>ÖZ</t>
-  </si>
-  <si>
-    <t>SEMA</t>
-  </si>
-  <si>
-    <t>ERCAN</t>
-  </si>
-  <si>
-    <t>DUYGU DOĞAN</t>
-  </si>
-  <si>
-    <t>GÜZELGÜN</t>
-  </si>
-  <si>
-    <t>15.06.2026 (2)</t>
   </si>
 </sst>
 </file>
@@ -1290,7 +1140,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V45"/>
+  <dimension ref="A1:V19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" style="29" customWidth="1"/>
@@ -1349,924 +1199,118 @@
         <v>3</v>
       </c>
       <c r="M1" s="27" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="N1" s="27" t="s">
         <v>3</v>
       </c>
       <c r="O1" s="27" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P1" s="27" t="s">
         <v>3</v>
       </c>
       <c r="Q1" s="27" t="s">
+        <v>9</v>
+      </c>
+      <c r="R1" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="R1" s="27" t="s">
+      <c r="S1" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="S1" s="27" t="s">
+      <c r="T1" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="T1" s="27" t="s">
+      <c r="U1" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="U1" s="27" t="s">
-        <v>14</v>
-      </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A2" s="29" t="s">
-        <v>176</v>
-      </c>
-      <c r="B2" s="29" t="s">
-        <v>177</v>
-      </c>
-      <c r="C2" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D2" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E2" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F2" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G2" s="30" t="s">
-        <v>224</v>
-      </c>
-      <c r="H2" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I2" s="30"/>
-      <c r="J2" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="Q2" s="30"/>
-      <c r="R2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="G2" s="30"/>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A3" s="29" t="s">
-        <v>178</v>
-      </c>
-      <c r="B3" s="29" t="s">
-        <v>179</v>
-      </c>
-      <c r="C3" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D3" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E3" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F3" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G3" s="30" t="s">
-        <v>224</v>
-      </c>
-      <c r="H3" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="J3" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="Q3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="G3" s="30"/>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A4" s="29" t="s">
-        <v>180</v>
-      </c>
-      <c r="B4" s="29" t="s">
-        <v>181</v>
-      </c>
-      <c r="C4" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D4" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E4" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F4" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G4" s="30" t="s">
-        <v>224</v>
-      </c>
-      <c r="H4" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I4" s="30"/>
-      <c r="J4" s="29" t="s">
-        <v>222</v>
-      </c>
+      <c r="C4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="G4" s="30"/>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A5" s="29" t="s">
-        <v>182</v>
-      </c>
-      <c r="B5" s="29" t="s">
-        <v>183</v>
-      </c>
-      <c r="C5" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D5" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E5" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F5" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G5" s="30" t="s">
-        <v>224</v>
-      </c>
-      <c r="H5" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I5" s="30"/>
-      <c r="J5" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="Q5" s="30"/>
-      <c r="R5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="E5" s="30"/>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A6" s="29" t="s">
-        <v>184</v>
-      </c>
-      <c r="B6" s="29" t="s">
-        <v>185</v>
-      </c>
-      <c r="C6" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D6" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E6" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F6" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G6" s="30" t="s">
-        <v>224</v>
-      </c>
-      <c r="H6" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I6" s="30"/>
-      <c r="J6" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="Q6" s="30"/>
-      <c r="R6" s="30"/>
+      <c r="C6" s="30"/>
+      <c r="E6" s="30"/>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A7" s="29" t="s">
-        <v>186</v>
-      </c>
-      <c r="B7" s="29" t="s">
-        <v>187</v>
-      </c>
-      <c r="C7" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D7" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E7" s="30" t="s">
-        <v>224</v>
-      </c>
-      <c r="F7" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G7" s="30"/>
-      <c r="H7" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I7" s="30"/>
-      <c r="J7" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="K7" s="30"/>
-      <c r="Q7" s="30"/>
-      <c r="R7" s="30"/>
-      <c r="S7" s="30"/>
-      <c r="T7" s="30"/>
+      <c r="C7" s="30"/>
+      <c r="E7" s="30"/>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A8" s="29" t="s">
-        <v>188</v>
-      </c>
-      <c r="B8" s="29" t="s">
-        <v>189</v>
-      </c>
-      <c r="C8" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D8" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E8" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F8" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G8" s="30" t="s">
-        <v>224</v>
-      </c>
-      <c r="H8" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I8" s="30"/>
-      <c r="J8" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="K8" s="30"/>
-      <c r="M8" s="30"/>
-      <c r="O8" s="30"/>
-      <c r="P8" s="30"/>
-      <c r="Q8" s="30"/>
-      <c r="R8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="E8" s="30"/>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A9" s="29" t="s">
-        <v>190</v>
-      </c>
-      <c r="B9" s="29" t="s">
-        <v>191</v>
-      </c>
-      <c r="C9" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D9" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E9" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F9" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G9" s="30" t="s">
-        <v>224</v>
-      </c>
-      <c r="H9" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="J9" s="29" t="s">
-        <v>222</v>
-      </c>
+      <c r="C9" s="30"/>
+      <c r="E9" s="30"/>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A10" s="29" t="s">
-        <v>192</v>
-      </c>
-      <c r="B10" s="29" t="s">
-        <v>193</v>
-      </c>
-      <c r="C10" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D10" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E10" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F10" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G10" s="30"/>
-      <c r="H10" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="J10" s="29" t="s">
-        <v>222</v>
-      </c>
+      <c r="C10" s="30"/>
+      <c r="E10" s="30"/>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A11" s="29" t="s">
-        <v>194</v>
-      </c>
-      <c r="B11" s="29" t="s">
-        <v>223</v>
-      </c>
-      <c r="C11" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D11" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E11" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F11" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G11" s="30">
-        <v>46188</v>
-      </c>
-      <c r="H11" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I11" s="30" t="s">
-        <v>224</v>
-      </c>
-      <c r="J11" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="Q11" s="30"/>
-      <c r="R11" s="30"/>
+      <c r="C11" s="30"/>
+      <c r="E11" s="30"/>
+      <c r="G11" s="30"/>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A12" s="29" t="s">
-        <v>195</v>
-      </c>
-      <c r="B12" s="29" t="s">
-        <v>196</v>
-      </c>
-      <c r="C12" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D12" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E12" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F12" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G12" s="30">
-        <v>46188</v>
-      </c>
-      <c r="H12" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I12" s="29" t="s">
-        <v>224</v>
-      </c>
-      <c r="J12" s="29" t="s">
-        <v>222</v>
-      </c>
+      <c r="A12" s="31"/>
+      <c r="B12" s="31"/>
+      <c r="C12" s="30"/>
+      <c r="E12" s="30"/>
+      <c r="G12" s="30"/>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A13" s="29" t="s">
-        <v>197</v>
-      </c>
-      <c r="B13" s="29" t="s">
-        <v>198</v>
-      </c>
-      <c r="C13" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D13" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E13" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F13" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G13" s="30" t="s">
-        <v>224</v>
-      </c>
-      <c r="H13" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="J13" s="29" t="s">
-        <v>222</v>
-      </c>
+      <c r="A13" s="31"/>
+      <c r="B13" s="31"/>
+      <c r="C13" s="30"/>
+      <c r="E13" s="30"/>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A14" s="29" t="s">
-        <v>199</v>
-      </c>
-      <c r="B14" s="29" t="s">
-        <v>200</v>
-      </c>
-      <c r="C14" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D14" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E14" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F14" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G14" s="30">
-        <v>46188</v>
-      </c>
-      <c r="H14" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I14" s="30" t="s">
-        <v>224</v>
-      </c>
-      <c r="J14" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="K14" s="30"/>
-      <c r="Q14" s="30"/>
-      <c r="R14" s="30"/>
-      <c r="S14" s="30"/>
+      <c r="A14" s="31"/>
+      <c r="B14" s="31"/>
+      <c r="C14" s="30"/>
+      <c r="E14" s="30"/>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A15" s="29" t="s">
-        <v>201</v>
-      </c>
-      <c r="B15" s="29" t="s">
-        <v>200</v>
-      </c>
-      <c r="C15" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D15" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E15" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F15" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G15" s="30">
-        <v>46188</v>
-      </c>
-      <c r="H15" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I15" s="29" t="s">
-        <v>224</v>
-      </c>
-      <c r="J15" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="K15" s="30"/>
-      <c r="Q15" s="30"/>
-      <c r="R15" s="30"/>
-      <c r="S15" s="30"/>
-      <c r="T15" s="30"/>
+      <c r="A15" s="31"/>
+      <c r="B15" s="31"/>
+      <c r="C15" s="30"/>
+      <c r="E15" s="30"/>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A16" s="29" t="s">
-        <v>202</v>
-      </c>
-      <c r="B16" s="29" t="s">
-        <v>203</v>
-      </c>
-      <c r="C16" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D16" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E16" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F16" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G16" s="29" t="s">
-        <v>224</v>
-      </c>
-      <c r="H16" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="J16" s="29" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A17" s="29" t="s">
-        <v>204</v>
-      </c>
-      <c r="B17" s="29" t="s">
-        <v>205</v>
-      </c>
-      <c r="C17" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D17" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E17" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F17" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G17" s="30">
-        <v>46188</v>
-      </c>
-      <c r="H17" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I17" s="29" t="s">
-        <v>224</v>
-      </c>
-      <c r="J17" s="29" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A18" s="29" t="s">
-        <v>206</v>
-      </c>
-      <c r="B18" s="29" t="s">
-        <v>207</v>
-      </c>
-      <c r="C18" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D18" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E18" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F18" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G18" s="30">
-        <v>46188</v>
-      </c>
-      <c r="H18" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I18" s="30" t="s">
-        <v>224</v>
-      </c>
-      <c r="J18" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="K18" s="30"/>
-      <c r="O18" s="30"/>
-      <c r="Q18" s="30"/>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A19" s="29" t="s">
-        <v>208</v>
-      </c>
-      <c r="B19" s="29" t="s">
-        <v>209</v>
-      </c>
-      <c r="C19" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D19" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E19" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F19" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G19" s="30">
-        <v>46188</v>
-      </c>
-      <c r="H19" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I19" s="29" t="s">
-        <v>224</v>
-      </c>
-      <c r="J19" s="29" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A20" s="29" t="s">
-        <v>210</v>
-      </c>
-      <c r="B20" s="29" t="s">
-        <v>209</v>
-      </c>
-      <c r="C20" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D20" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E20" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F20" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G20" s="30">
-        <v>46188</v>
-      </c>
-      <c r="H20" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I20" s="29" t="s">
-        <v>224</v>
-      </c>
-      <c r="J20" s="29" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A21" s="29" t="s">
-        <v>211</v>
-      </c>
-      <c r="B21" s="29" t="s">
-        <v>212</v>
-      </c>
-      <c r="C21" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D21" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E21" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F21" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G21" s="30">
-        <v>46188</v>
-      </c>
-      <c r="H21" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I21" s="29" t="s">
-        <v>224</v>
-      </c>
-      <c r="J21" s="29" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A22" s="29" t="s">
-        <v>213</v>
-      </c>
-      <c r="B22" s="29" t="s">
-        <v>214</v>
-      </c>
-      <c r="C22" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D22" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E22" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F22" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G22" s="30">
-        <v>46188</v>
-      </c>
-      <c r="H22" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I22" s="29" t="s">
-        <v>224</v>
-      </c>
-      <c r="J22" s="29" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A23" s="29" t="s">
-        <v>206</v>
-      </c>
-      <c r="B23" s="29" t="s">
-        <v>215</v>
-      </c>
-      <c r="C23" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D23" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E23" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F23" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G23" s="30">
-        <v>46188</v>
-      </c>
-      <c r="H23" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I23" s="29" t="s">
-        <v>224</v>
-      </c>
-      <c r="J23" s="29" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="29" t="s">
-        <v>216</v>
-      </c>
-      <c r="B24" s="29" t="s">
-        <v>217</v>
-      </c>
-      <c r="C24" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D24" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E24" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F24" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G24" s="30">
-        <v>46188</v>
-      </c>
-      <c r="H24" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I24" s="30" t="s">
-        <v>224</v>
-      </c>
-      <c r="J24" s="29" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A25" s="29" t="s">
-        <v>218</v>
-      </c>
-      <c r="B25" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="C25" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D25" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E25" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F25" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G25" s="30">
-        <v>46188</v>
-      </c>
-      <c r="H25" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I25" s="29" t="s">
-        <v>224</v>
-      </c>
-      <c r="J25" s="29" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A26" s="29" t="s">
-        <v>220</v>
-      </c>
-      <c r="B26" s="29" t="s">
-        <v>221</v>
-      </c>
-      <c r="C26" s="30">
-        <v>46190</v>
-      </c>
-      <c r="D26" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E26" s="30">
-        <v>46189</v>
-      </c>
-      <c r="F26" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="G26" s="30">
-        <v>46188</v>
-      </c>
-      <c r="H26" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I26" s="29" t="s">
-        <v>224</v>
-      </c>
-      <c r="J26" s="29" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="C27" s="30"/>
-      <c r="E27" s="30"/>
-      <c r="G27" s="30"/>
-    </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="C28" s="30"/>
-      <c r="E28" s="30"/>
-      <c r="G28" s="30"/>
-    </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="C29" s="30"/>
-      <c r="E29" s="30"/>
-      <c r="G29" s="30"/>
-    </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="C30" s="30"/>
-      <c r="E30" s="30"/>
-      <c r="G30" s="30"/>
-    </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="C31" s="30"/>
-      <c r="E31" s="30"/>
-    </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="C32" s="30"/>
-      <c r="E32" s="30"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C33" s="30"/>
-      <c r="E33" s="30"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C34" s="30"/>
-      <c r="E34" s="30"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C35" s="30"/>
-      <c r="E35" s="30"/>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C36" s="30"/>
-      <c r="E36" s="30"/>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C37" s="30"/>
-      <c r="E37" s="30"/>
-      <c r="G37" s="30"/>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A38" s="31"/>
-      <c r="B38" s="31"/>
-      <c r="C38" s="30"/>
-      <c r="E38" s="30"/>
-      <c r="G38" s="30"/>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A39" s="31"/>
-      <c r="B39" s="31"/>
-      <c r="C39" s="30"/>
-      <c r="E39" s="30"/>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A40" s="31"/>
-      <c r="B40" s="31"/>
-      <c r="C40" s="30"/>
-      <c r="E40" s="30"/>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A41" s="31"/>
-      <c r="B41" s="31"/>
-      <c r="C41" s="30"/>
-      <c r="E41" s="30"/>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C42" s="30"/>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C43" s="30"/>
-      <c r="G43" s="30"/>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C44" s="30"/>
-      <c r="E44" s="30"/>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C45" s="30"/>
+      <c r="C16" s="30"/>
+    </row>
+    <row r="17" spans="3:7" x14ac:dyDescent="0.3">
+      <c r="C17" s="30"/>
+      <c r="G17" s="30"/>
+    </row>
+    <row r="18" spans="3:7" x14ac:dyDescent="0.3">
+      <c r="C18" s="30"/>
+      <c r="E18" s="30"/>
+    </row>
+    <row r="19" spans="3:7" x14ac:dyDescent="0.3">
+      <c r="C19" s="30"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U29" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:U3" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2326,22 +1370,22 @@
         <v>3</v>
       </c>
       <c r="K1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
@@ -2728,22 +1772,22 @@
         <v>3</v>
       </c>
       <c r="K1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
@@ -3147,22 +2191,22 @@
         <v>3</v>
       </c>
       <c r="K1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
@@ -3279,22 +2323,22 @@
         <v>3</v>
       </c>
       <c r="K1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
@@ -3411,22 +2455,22 @@
         <v>3</v>
       </c>
       <c r="K1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
@@ -3885,22 +2929,22 @@
         <v>3</v>
       </c>
       <c r="K1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
@@ -4592,22 +3636,22 @@
         <v>3</v>
       </c>
       <c r="K1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
@@ -4703,19 +3747,19 @@
         <v>3</v>
       </c>
       <c r="M1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="N1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
@@ -4910,22 +3954,22 @@
         <v>3</v>
       </c>
       <c r="K1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
@@ -5085,49 +4129,49 @@
         <v>3</v>
       </c>
       <c r="M1" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N1" s="11" t="s">
         <v>3</v>
       </c>
       <c r="O1" s="11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="P1" s="11" t="s">
         <v>3</v>
       </c>
       <c r="Q1" s="11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="R1" s="11" t="s">
         <v>3</v>
       </c>
       <c r="S1" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="T1" s="11" t="s">
         <v>3</v>
       </c>
       <c r="U1" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="V1" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="V1" s="11" t="s">
+      <c r="W1" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="W1" s="11" t="s">
+      <c r="X1" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="X1" s="11" t="s">
+      <c r="Y1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Z1" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="Z1" s="25" t="s">
-        <v>15</v>
-      </c>
       <c r="AA1" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.3">
@@ -5502,42 +4546,42 @@
         <v>3</v>
       </c>
       <c r="K1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>21</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>22</v>
       </c>
       <c r="C2" s="5">
         <v>45771</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E2" s="5">
         <v>45772</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G2" s="5">
         <v>45776</v>
@@ -5554,22 +4598,22 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>24</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>25</v>
       </c>
       <c r="C3" s="5">
         <v>45771</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E3" s="5">
         <v>45819</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
@@ -5583,22 +4627,22 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="C4" s="5">
         <v>45771</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E4" s="5">
         <v>45785</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -5613,22 +4657,22 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>28</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>29</v>
       </c>
       <c r="C5" s="5">
         <v>45768</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E5" s="5">
         <v>45776</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G5" s="5">
         <v>45777</v>
@@ -5645,22 +4689,22 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>31</v>
       </c>
       <c r="C6" s="5">
         <v>45768</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E6" s="5">
         <v>45771</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -5675,20 +4719,20 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>32</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>33</v>
       </c>
       <c r="C7" s="5">
         <v>45768</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E7" s="4"/>
       <c r="F7" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -5703,22 +4747,22 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>35</v>
       </c>
       <c r="C8" s="5">
         <v>45768</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E8" s="5">
         <v>45769</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G8" s="5">
         <v>45771</v>
@@ -5735,22 +4779,22 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>37</v>
       </c>
       <c r="C9" s="5">
         <v>45768</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E9" s="5">
         <v>45769</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G9" s="5">
         <v>45772</v>
@@ -5767,22 +4811,22 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>38</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="C10" s="5">
         <v>45768</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E10" s="5">
         <v>45772</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G10" s="5">
         <v>45776</v>
@@ -5799,22 +4843,22 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>41</v>
       </c>
       <c r="C11" s="5">
         <v>45768</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E11" s="5">
         <v>45775</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -5829,22 +4873,22 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>42</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>43</v>
       </c>
       <c r="C12" s="5">
         <v>45769</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E12" s="5">
         <v>45772</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -5859,22 +4903,22 @@
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>44</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>45</v>
       </c>
       <c r="C13" s="5">
         <v>45769</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E13" s="5">
         <v>45772</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G13" s="5">
         <v>45775</v>
@@ -5891,22 +4935,22 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>46</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>47</v>
       </c>
       <c r="C14" s="5">
         <v>45769</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E14" s="5">
         <v>45771</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G14" s="5">
         <v>45779</v>
@@ -5923,22 +4967,22 @@
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>48</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>49</v>
       </c>
       <c r="C15" s="5">
         <v>45769</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E15" s="5">
         <v>45789</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -5953,20 +4997,20 @@
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>50</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>51</v>
       </c>
       <c r="C16" s="5">
         <v>45769</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E16" s="4"/>
       <c r="F16" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -5981,22 +5025,22 @@
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>53</v>
       </c>
       <c r="C17" s="5">
         <v>45769</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E17" s="5">
         <v>45776</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G17" s="5">
         <v>45786</v>
@@ -6013,22 +5057,22 @@
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>54</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>55</v>
       </c>
       <c r="C18" s="5">
         <v>45769</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E18" s="5">
         <v>45792</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -6043,22 +5087,22 @@
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>56</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>57</v>
       </c>
       <c r="C19" s="5">
         <v>45769</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E19" s="5">
         <v>45772</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
@@ -6073,22 +5117,22 @@
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>58</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>59</v>
       </c>
       <c r="C20" s="5">
         <v>45769</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E20" s="5">
         <v>45772</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G20" s="5">
         <v>45777</v>
@@ -6105,22 +5149,22 @@
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>60</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>61</v>
       </c>
       <c r="C21" s="5">
         <v>45769</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E21" s="5">
         <v>45775</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -6135,22 +5179,22 @@
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C22" s="5">
         <v>45771</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E22" s="5">
         <v>45772</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G22" s="5">
         <v>45789</v>
@@ -6167,22 +5211,22 @@
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B23" s="4" t="s">
         <v>63</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>64</v>
       </c>
       <c r="C23" s="5">
         <v>45771</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E23" s="5">
         <v>45775</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
@@ -6197,22 +5241,22 @@
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B24" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>66</v>
       </c>
       <c r="C24" s="5">
         <v>45771</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E24" s="5">
         <v>45775</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G24" s="5">
         <v>45789</v>
@@ -6229,22 +5273,22 @@
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B25" s="4" t="s">
         <v>67</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>68</v>
       </c>
       <c r="C25" s="5">
         <v>45771</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E25" s="5">
         <v>45772</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -6259,22 +5303,22 @@
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B26" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>70</v>
       </c>
       <c r="C26" s="5">
         <v>45771</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E26" s="5">
         <v>45772</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G26" s="5">
         <v>45775</v>
@@ -6291,22 +5335,22 @@
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>71</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>72</v>
       </c>
       <c r="C27" s="5">
         <v>45771</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E27" s="5">
         <v>45777</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G27" s="5">
         <v>45785</v>
@@ -6323,20 +5367,20 @@
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B28" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>74</v>
       </c>
       <c r="C28" s="5">
         <v>45771</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E28" s="4"/>
       <c r="F28" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
@@ -6351,22 +5395,22 @@
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B29" s="4" t="s">
         <v>75</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>76</v>
       </c>
       <c r="C29" s="5">
         <v>45771</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E29" s="5">
         <v>45777</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
@@ -6381,22 +5425,22 @@
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B30" s="4" t="s">
         <v>77</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>78</v>
       </c>
       <c r="C30" s="5">
         <v>45771</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E30" s="5">
         <v>45777</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G30" s="5">
         <v>45785</v>
@@ -6413,22 +5457,22 @@
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C31" s="5">
         <v>45771</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E31" s="5">
         <v>45777</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G31" s="5">
         <v>45785</v>
@@ -6445,20 +5489,20 @@
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B32" s="4" t="s">
         <v>80</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>81</v>
       </c>
       <c r="C32" s="5">
         <v>45771</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E32" s="4"/>
       <c r="F32" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -6473,22 +5517,22 @@
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B33" s="4" t="s">
         <v>82</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>83</v>
       </c>
       <c r="C33" s="5">
         <v>45769</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E33" s="5">
         <v>45771</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G33" s="5">
         <v>45772</v>
@@ -6505,22 +5549,22 @@
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B34" s="4" t="s">
         <v>84</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>85</v>
       </c>
       <c r="C34" s="5">
         <v>45771</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E34" s="5">
         <v>45776</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G34" s="5">
         <v>45777</v>
@@ -6537,22 +5581,22 @@
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B35" s="4" t="s">
         <v>86</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>87</v>
       </c>
       <c r="C35" s="5">
         <v>45771</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E35" s="5">
         <v>45775</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G35" s="5">
         <v>45776</v>
@@ -6569,22 +5613,22 @@
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B36" s="4" t="s">
         <v>88</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>89</v>
       </c>
       <c r="C36" s="5">
         <v>45768</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E36" s="5">
         <v>45771</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G36" s="5">
         <v>45775</v>
@@ -6601,22 +5645,22 @@
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B37" s="4" t="s">
         <v>90</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>91</v>
       </c>
       <c r="C37" s="5">
         <v>45771</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E37" s="5">
         <v>45792</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
@@ -6631,20 +5675,20 @@
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B38" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="C38" s="5">
         <v>45776</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E38" s="4"/>
       <c r="F38" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
@@ -6659,22 +5703,22 @@
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C39" s="5">
         <v>45776</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E39" s="5">
         <v>45789</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -6689,20 +5733,20 @@
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C40" s="5">
         <v>45776</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E40" s="4"/>
       <c r="F40" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
@@ -6717,22 +5761,22 @@
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C41" s="5">
         <v>45776</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E41" s="5">
         <v>45779</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
@@ -6747,22 +5791,22 @@
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B42" s="6" t="s">
         <v>95</v>
-      </c>
-      <c r="B42" s="6" t="s">
-        <v>96</v>
       </c>
       <c r="C42" s="5">
         <v>45769</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E42" s="5">
         <v>45772</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G42" s="5">
         <v>45776</v>
@@ -6779,22 +5823,22 @@
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B43" s="4" t="s">
         <v>97</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>98</v>
       </c>
       <c r="C43" s="5">
         <v>45776</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E43" s="5">
         <v>45791</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G43" s="5">
         <v>45792</v>
@@ -6810,20 +5854,20 @@
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B44" s="4" t="s">
         <v>99</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>100</v>
       </c>
       <c r="C44" s="5">
         <v>45771</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E44" s="4"/>
       <c r="F44" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
@@ -6838,22 +5882,22 @@
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B45" s="4" t="s">
         <v>101</v>
-      </c>
-      <c r="B45" s="4" t="s">
-        <v>102</v>
       </c>
       <c r="C45" s="5">
         <v>45771</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E45" s="5">
         <v>45772</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G45" s="5">
         <v>45776</v>
@@ -6870,22 +5914,22 @@
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C46" s="5">
         <v>45771</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E46" s="5">
         <v>45789</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -6900,22 +5944,22 @@
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C47" s="5">
         <v>45771</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E47" s="5">
         <v>45775</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G47" s="5">
         <v>45798</v>
@@ -6932,22 +5976,22 @@
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B48" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="B48" s="4" t="s">
-        <v>106</v>
       </c>
       <c r="C48" s="5">
         <v>45772</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E48" s="5">
         <v>45775</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G48" s="5">
         <v>45786</v>
@@ -6964,22 +6008,22 @@
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A49" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C49" s="5">
         <v>45772</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E49" s="5">
         <v>45777</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
@@ -6994,20 +6038,20 @@
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B50" s="4" t="s">
         <v>107</v>
-      </c>
-      <c r="B50" s="4" t="s">
-        <v>108</v>
       </c>
       <c r="C50" s="5">
         <v>45772</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E50" s="4"/>
       <c r="F50" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
@@ -7022,22 +6066,22 @@
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A51" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B51" s="4" t="s">
         <v>109</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>110</v>
       </c>
       <c r="C51" s="5">
         <v>45772</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E51" s="5">
         <v>45779</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -7052,22 +6096,22 @@
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B52" s="4" t="s">
         <v>111</v>
-      </c>
-      <c r="B52" s="4" t="s">
-        <v>112</v>
       </c>
       <c r="C52" s="5">
         <v>45772</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E52" s="5">
         <v>45775</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G52" s="5">
         <v>45786</v>
@@ -7084,22 +6128,22 @@
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A53" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C53" s="5">
         <v>45772</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E53" s="5">
         <v>45785</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
@@ -7114,22 +6158,22 @@
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B54" s="4" t="s">
         <v>114</v>
-      </c>
-      <c r="B54" s="4" t="s">
-        <v>115</v>
       </c>
       <c r="C54" s="5">
         <v>45772</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E54" s="5">
         <v>45786</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
@@ -7144,20 +6188,20 @@
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A55" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B55" s="4" t="s">
         <v>116</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>117</v>
       </c>
       <c r="C55" s="5">
         <v>45772</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E55" s="4"/>
       <c r="F55" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
@@ -7172,22 +6216,22 @@
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B56" s="4" t="s">
         <v>118</v>
-      </c>
-      <c r="B56" s="4" t="s">
-        <v>119</v>
       </c>
       <c r="C56" s="5">
         <v>45772</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E56" s="5">
         <v>45819</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G56" s="4"/>
       <c r="H56" s="4"/>
@@ -7202,20 +6246,20 @@
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C57" s="5">
         <v>45772</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E57" s="4"/>
       <c r="F57" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G57" s="4"/>
       <c r="H57" s="4"/>
@@ -7230,22 +6274,22 @@
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B58" s="4" t="s">
         <v>121</v>
-      </c>
-      <c r="B58" s="4" t="s">
-        <v>122</v>
       </c>
       <c r="C58" s="5">
         <v>45772</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E58" s="5">
         <v>45775</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
@@ -7260,20 +6304,20 @@
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C59" s="5">
         <v>45772</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E59" s="4"/>
       <c r="F59" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G59" s="4"/>
       <c r="H59" s="4"/>
@@ -7288,22 +6332,22 @@
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B60" s="4" t="s">
         <v>124</v>
-      </c>
-      <c r="B60" s="4" t="s">
-        <v>125</v>
       </c>
       <c r="C60" s="5">
         <v>45772</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E60" s="5">
         <v>45775</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
@@ -7318,22 +6362,22 @@
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="B61" s="4" t="s">
         <v>126</v>
-      </c>
-      <c r="B61" s="4" t="s">
-        <v>127</v>
       </c>
       <c r="C61" s="5">
         <v>45772</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E61" s="5">
         <v>45789</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G61" s="4"/>
       <c r="H61" s="4"/>
@@ -7348,22 +6392,22 @@
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B62" s="4" t="s">
         <v>128</v>
-      </c>
-      <c r="B62" s="4" t="s">
-        <v>129</v>
       </c>
       <c r="C62" s="5">
         <v>45772</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E62" s="5">
         <v>45775</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G62" s="5">
         <v>45789</v>
@@ -7380,22 +6424,22 @@
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B63" s="4" t="s">
         <v>130</v>
-      </c>
-      <c r="B63" s="4" t="s">
-        <v>131</v>
       </c>
       <c r="C63" s="5">
         <v>45775</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E63" s="5">
         <v>45789</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
@@ -7410,20 +6454,20 @@
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C64" s="5">
         <v>45775</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E64" s="4"/>
       <c r="F64" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G64" s="4"/>
       <c r="H64" s="4"/>
@@ -7438,20 +6482,20 @@
     </row>
     <row r="65" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A65" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C65" s="5">
         <v>45775</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E65" s="4"/>
       <c r="F65" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G65" s="4"/>
       <c r="H65" s="4"/>
@@ -7466,22 +6510,22 @@
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B66" s="4" t="s">
         <v>134</v>
-      </c>
-      <c r="B66" s="4" t="s">
-        <v>135</v>
       </c>
       <c r="C66" s="5">
         <v>45775</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E66" s="5">
         <v>45786</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G66" s="4"/>
       <c r="H66" s="4"/>
@@ -7496,22 +6540,22 @@
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A67" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B67" s="4" t="s">
         <v>136</v>
-      </c>
-      <c r="B67" s="4" t="s">
-        <v>137</v>
       </c>
       <c r="C67" s="5">
         <v>45776</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E67" s="5">
         <v>45777</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G67" s="5">
         <v>45779</v>
@@ -7528,20 +6572,20 @@
     </row>
     <row r="68" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C68" s="5">
         <v>45776</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E68" s="5"/>
       <c r="F68" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G68" s="4"/>
       <c r="H68" s="4"/>
@@ -7556,20 +6600,20 @@
     </row>
     <row r="69" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C69" s="5">
         <v>45776</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E69" s="4"/>
       <c r="F69" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G69" s="4"/>
       <c r="H69" s="4"/>
@@ -7584,20 +6628,20 @@
     </row>
     <row r="70" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C70" s="5">
         <v>45776</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E70" s="4"/>
       <c r="F70" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G70" s="4"/>
       <c r="H70" s="4"/>
@@ -7612,20 +6656,20 @@
     </row>
     <row r="71" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A71" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C71" s="5">
         <v>45776</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E71" s="4"/>
       <c r="F71" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G71" s="4"/>
       <c r="H71" s="4"/>
@@ -7640,22 +6684,22 @@
     </row>
     <row r="72" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B72" s="4" t="s">
         <v>142</v>
-      </c>
-      <c r="B72" s="4" t="s">
-        <v>143</v>
       </c>
       <c r="C72" s="5">
         <v>45769</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E72" s="5">
         <v>45772</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G72" s="5">
         <v>45776</v>
@@ -7672,22 +6716,22 @@
     </row>
     <row r="73" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B73" s="4" t="s">
         <v>144</v>
-      </c>
-      <c r="B73" s="4" t="s">
-        <v>145</v>
       </c>
       <c r="C73" s="5">
         <v>45771</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E73" s="5">
         <v>45776</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G73" s="4"/>
       <c r="H73" s="4"/>
@@ -7702,22 +6746,22 @@
     </row>
     <row r="74" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C74" s="5">
         <v>45775</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E74" s="5">
         <v>45776</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G74" s="5">
         <v>45786</v>
@@ -7734,22 +6778,22 @@
     </row>
     <row r="75" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A75" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B75" s="4" t="s">
         <v>147</v>
-      </c>
-      <c r="B75" s="4" t="s">
-        <v>148</v>
       </c>
       <c r="C75" s="5">
         <v>45776</v>
       </c>
       <c r="D75" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E75" s="5">
         <v>45792</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G75" s="4"/>
       <c r="H75" s="4"/>
@@ -7764,20 +6808,20 @@
     </row>
     <row r="76" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B76" s="4" t="s">
         <v>149</v>
-      </c>
-      <c r="B76" s="4" t="s">
-        <v>150</v>
       </c>
       <c r="C76" s="5">
         <v>45776</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E76" s="4"/>
       <c r="F76" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G76" s="4"/>
       <c r="H76" s="4"/>
@@ -7792,22 +6836,22 @@
     </row>
     <row r="77" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A77" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C77" s="5">
         <v>45776</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E77" s="5">
         <v>45792</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G77" s="4"/>
       <c r="H77" s="4"/>
@@ -7822,22 +6866,22 @@
     </row>
     <row r="78" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B78" s="4" t="s">
         <v>152</v>
-      </c>
-      <c r="B78" s="4" t="s">
-        <v>153</v>
       </c>
       <c r="C78" s="5">
         <v>45776</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E78" s="5">
         <v>45792</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G78" s="5">
         <v>45819</v>
@@ -7854,20 +6898,20 @@
     </row>
     <row r="79" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="B79" s="4" t="s">
         <v>154</v>
-      </c>
-      <c r="B79" s="4" t="s">
-        <v>155</v>
       </c>
       <c r="C79" s="5">
         <v>45776</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E79" s="4"/>
       <c r="F79" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G79" s="4"/>
       <c r="H79" s="4"/>
@@ -7882,22 +6926,22 @@
     </row>
     <row r="80" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B80" s="4" t="s">
         <v>156</v>
-      </c>
-      <c r="B80" s="4" t="s">
-        <v>157</v>
       </c>
       <c r="C80" s="5">
         <v>45771</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E80" s="5">
         <v>45776</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G80" s="4"/>
       <c r="H80" s="4"/>
@@ -7912,22 +6956,22 @@
     </row>
     <row r="81" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="B81" s="4" t="s">
         <v>158</v>
-      </c>
-      <c r="B81" s="4" t="s">
-        <v>159</v>
       </c>
       <c r="C81" s="5">
         <v>45769</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E81" s="5">
         <v>45776</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G81" s="5">
         <v>45792</v>
@@ -7944,22 +6988,22 @@
     </row>
     <row r="82" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C82" s="5">
         <v>45777</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E82" s="5">
         <v>45779</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G82" s="5">
         <v>45786</v>
@@ -7976,19 +7020,19 @@
     </row>
     <row r="83" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C83" s="5">
         <v>45777</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G83" s="4"/>
       <c r="H83" s="4"/>
@@ -8003,22 +7047,22 @@
     </row>
     <row r="84" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A84" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="B84" s="4" t="s">
         <v>162</v>
-      </c>
-      <c r="B84" s="4" t="s">
-        <v>163</v>
       </c>
       <c r="C84" s="5">
         <v>45784</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E84" s="5">
         <v>45791</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G84" s="4"/>
       <c r="H84" s="4"/>
@@ -8033,20 +7077,20 @@
     </row>
     <row r="85" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A85" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C85" s="5">
         <v>45784</v>
       </c>
       <c r="D85" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E85" s="4"/>
       <c r="F85" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G85" s="4"/>
       <c r="H85" s="4"/>
@@ -8061,20 +7105,20 @@
     </row>
     <row r="86" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A86" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="B86" s="4" t="s">
         <v>165</v>
-      </c>
-      <c r="B86" s="4" t="s">
-        <v>166</v>
       </c>
       <c r="C86" s="5">
         <v>45784</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E86" s="4"/>
       <c r="F86" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G86" s="4"/>
       <c r="H86" s="4"/>
@@ -8089,22 +7133,22 @@
     </row>
     <row r="87" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B87" s="4" t="s">
         <v>167</v>
-      </c>
-      <c r="B87" s="4" t="s">
-        <v>168</v>
       </c>
       <c r="C87" s="5">
         <v>45784</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E87" s="5">
         <v>45791</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G87" s="4"/>
       <c r="H87" s="4"/>
@@ -8119,20 +7163,20 @@
     </row>
     <row r="88" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A88" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B88" s="4" t="s">
         <v>169</v>
-      </c>
-      <c r="B88" s="4" t="s">
-        <v>170</v>
       </c>
       <c r="C88" s="5">
         <v>45785</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E88" s="4"/>
       <c r="F88" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G88" s="4"/>
       <c r="H88" s="4"/>
@@ -8147,22 +7191,22 @@
     </row>
     <row r="89" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A89" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B89" s="4" t="s">
         <v>171</v>
-      </c>
-      <c r="B89" s="4" t="s">
-        <v>172</v>
       </c>
       <c r="C89" s="5">
         <v>45789</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E89" s="5">
         <v>45792</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G89" s="4"/>
       <c r="H89" s="4"/>
@@ -8177,20 +7221,20 @@
     </row>
     <row r="90" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A90" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C90" s="5">
         <v>45819</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E90" s="4"/>
       <c r="F90" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G90" s="4"/>
       <c r="H90" s="4"/>
@@ -8205,20 +7249,20 @@
     </row>
     <row r="91" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A91" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B91" s="4" t="s">
         <v>174</v>
-      </c>
-      <c r="B91" s="4" t="s">
-        <v>175</v>
       </c>
       <c r="C91" s="5">
         <v>45819</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E91" s="4"/>
       <c r="F91" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G91" s="4"/>
       <c r="H91" s="4"/>
@@ -8236,11 +7280,11 @@
       <c r="B92" s="4"/>
       <c r="C92" s="4"/>
       <c r="D92" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E92" s="4"/>
       <c r="F92" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G92" s="4"/>
       <c r="H92" s="4"/>
@@ -8258,11 +7302,11 @@
       <c r="B93" s="4"/>
       <c r="C93" s="4"/>
       <c r="D93" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E93" s="4"/>
       <c r="F93" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G93" s="4"/>
       <c r="H93" s="4"/>
@@ -8280,11 +7324,11 @@
       <c r="B94" s="4"/>
       <c r="C94" s="4"/>
       <c r="D94" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E94" s="4"/>
       <c r="F94" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G94" s="4"/>
       <c r="H94" s="4"/>
@@ -8302,11 +7346,11 @@
       <c r="B95" s="4"/>
       <c r="C95" s="4"/>
       <c r="D95" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E95" s="4"/>
       <c r="F95" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G95" s="4"/>
       <c r="H95" s="4"/>
@@ -8324,11 +7368,11 @@
       <c r="B96" s="4"/>
       <c r="C96" s="4"/>
       <c r="D96" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E96" s="4"/>
       <c r="F96" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G96" s="4"/>
       <c r="H96" s="4"/>
@@ -8346,11 +7390,11 @@
       <c r="B97" s="4"/>
       <c r="C97" s="4"/>
       <c r="D97" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E97" s="4"/>
       <c r="F97" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G97" s="4"/>
       <c r="H97" s="4"/>
@@ -8368,11 +7412,11 @@
       <c r="B98" s="4"/>
       <c r="C98" s="4"/>
       <c r="D98" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E98" s="4"/>
       <c r="F98" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G98" s="4"/>
       <c r="H98" s="4"/>
@@ -8390,11 +7434,11 @@
       <c r="B99" s="4"/>
       <c r="C99" s="4"/>
       <c r="D99" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E99" s="4"/>
       <c r="F99" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G99" s="4"/>
       <c r="H99" s="4"/>
@@ -8412,11 +7456,11 @@
       <c r="B100" s="4"/>
       <c r="C100" s="4"/>
       <c r="D100" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E100" s="4"/>
       <c r="F100" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G100" s="4"/>
       <c r="H100" s="4"/>
@@ -8434,11 +7478,11 @@
       <c r="B101" s="4"/>
       <c r="C101" s="4"/>
       <c r="D101" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E101" s="4"/>
       <c r="F101" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G101" s="4"/>
       <c r="H101" s="4"/>
@@ -8456,11 +7500,11 @@
       <c r="B102" s="4"/>
       <c r="C102" s="4"/>
       <c r="D102" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E102" s="4"/>
       <c r="F102" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G102" s="4"/>
       <c r="H102" s="4"/>
@@ -8480,7 +7524,7 @@
       <c r="D103" s="4"/>
       <c r="E103" s="4"/>
       <c r="F103" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G103" s="4"/>
       <c r="H103" s="4"/>
@@ -10264,6 +9308,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d0e89180-09d0-4a61-9d87-e9890741df71">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="0a1727d5-2cd7-48d5-83a7-d4ed5f973127" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Belge" ma:contentTypeID="0x010100C9EC04EC2BEE9C48A0FBA194F70FAAE8" ma:contentTypeVersion="15" ma:contentTypeDescription="Yeni belge oluşturun." ma:contentTypeScope="" ma:versionID="afea4d98ca95f55432d1afcf39d2ed73">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d0e89180-09d0-4a61-9d87-e9890741df71" xmlns:ns3="0a1727d5-2cd7-48d5-83a7-d4ed5f973127" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ca2e74ded007f18db906e2ccd86cf64c" ns2:_="" ns3:_="">
     <xsd:import namespace="d0e89180-09d0-4a61-9d87-e9890741df71"/>
@@ -10498,17 +9553,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d0e89180-09d0-4a61-9d87-e9890741df71">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="0a1727d5-2cd7-48d5-83a7-d4ed5f973127" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -10519,6 +9563,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{728F81EF-DA50-48F9-BF25-6CC419B8F51F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d0e89180-09d0-4a61-9d87-e9890741df71"/>
+    <ds:schemaRef ds:uri="0a1727d5-2cd7-48d5-83a7-d4ed5f973127"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C5D477F-7D2B-487E-9BAC-E40D5BC1AD78}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10537,17 +9592,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{728F81EF-DA50-48F9-BF25-6CC419B8F51F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d0e89180-09d0-4a61-9d87-e9890741df71"/>
-    <ds:schemaRef ds:uri="0a1727d5-2cd7-48d5-83a7-d4ed5f973127"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5690AD69-5F77-485B-8CC9-BD5B85428455}">
   <ds:schemaRefs>

</xml_diff>